<commit_message>
feat: RekonKlasis export, REALISASI Dianggarkan, carryover anggaran; bersihkan file sampah
</commit_message>
<xml_diff>
--- a/data/MAPPING REKON.xlsx
+++ b/data/MAPPING REKON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\JONDRY\keuangan-app\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{905DC52C-3110-434F-9073-37F0E0ED2BFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A911FA64-9B1D-4D7F-86D3-850704CA7A59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{1172081E-8F43-4ADA-9126-2378305563B8}"/>
   </bookViews>
@@ -73,9 +73,6 @@
     <t xml:space="preserve">REALISASI PERBULAN / TAHUN </t>
   </si>
   <si>
-    <t>APB-G TA 2024</t>
-  </si>
-  <si>
     <t xml:space="preserve">BULAN </t>
   </si>
   <si>
@@ -194,6 +191,9 @@
   </si>
   <si>
     <t>Pnt Ny. O. Tapilaha</t>
+  </si>
+  <si>
+    <t>APB-G TA 2025</t>
   </si>
 </sst>
 </file>
@@ -295,7 +295,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -333,17 +333,6 @@
     </border>
     <border>
       <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -390,6 +379,211 @@
       </right>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -397,11 +591,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -415,77 +606,26 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -507,9 +647,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -527,9 +664,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -540,11 +674,126 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -582,9 +831,9 @@
       <sheetName val="RANCANGAN ANGGARAN 2026"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
       <sheetData sheetId="3">
         <row r="13">
           <cell r="C13">
@@ -813,13 +1062,13 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="7" refreshError="1"/>
+      <sheetData sheetId="8" refreshError="1"/>
+      <sheetData sheetId="9" refreshError="1"/>
+      <sheetData sheetId="10" refreshError="1"/>
+      <sheetData sheetId="11" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -1188,892 +1437,884 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="37"/>
+      <c r="J1" s="37"/>
     </row>
     <row r="2" spans="1:10" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
+      <c r="B2" s="37"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
+      <c r="G2" s="37"/>
+      <c r="H2" s="37"/>
+      <c r="I2" s="37"/>
+      <c r="J2" s="37"/>
     </row>
     <row r="3" spans="1:10" ht="18" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
+      <c r="B3" s="37"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="37"/>
+      <c r="G3" s="37"/>
+      <c r="H3" s="37"/>
+      <c r="I3" s="37"/>
+      <c r="J3" s="37"/>
     </row>
     <row r="4" spans="1:10" ht="18" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+    </row>
+    <row r="5" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="5" t="s">
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="J5" s="5" t="s">
+      <c r="J5" s="4" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="59" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="60" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="9"/>
+      <c r="C6" s="61"/>
+      <c r="D6" s="61"/>
+      <c r="E6" s="61"/>
+      <c r="F6" s="61"/>
+      <c r="G6" s="61"/>
+      <c r="H6" s="61"/>
+      <c r="I6" s="61"/>
+      <c r="J6" s="62"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="63" t="s">
+        <v>49</v>
+      </c>
+      <c r="B7" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="C7" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="D7" s="41"/>
+      <c r="E7" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="12"/>
-      <c r="E7" s="11" t="s">
+      <c r="F7" s="41"/>
+      <c r="G7" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="12"/>
-      <c r="G7" s="10" t="s">
+      <c r="H7" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="13" t="s">
+      <c r="I7" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="I7" s="14" t="s">
+      <c r="J7" s="64" t="s">
         <v>15</v>
       </c>
-      <c r="J7" s="14" t="s">
+    </row>
+    <row r="8" spans="1:10" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A8" s="65"/>
+      <c r="B8" s="39"/>
+      <c r="C8" s="5" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="15"/>
-      <c r="B8" s="15"/>
-      <c r="C8" s="16" t="s">
+      <c r="D8" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="E8" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" s="39"/>
+      <c r="H8" s="43"/>
+      <c r="I8" s="33"/>
+      <c r="J8" s="66"/>
+    </row>
+    <row r="9" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="67">
+        <v>1</v>
+      </c>
+      <c r="B9" s="68">
+        <v>2</v>
+      </c>
+      <c r="C9" s="68">
+        <v>3</v>
+      </c>
+      <c r="D9" s="68">
+        <v>4</v>
+      </c>
+      <c r="E9" s="69">
+        <v>5</v>
+      </c>
+      <c r="F9" s="69">
+        <v>6</v>
+      </c>
+      <c r="G9" s="69">
+        <v>7</v>
+      </c>
+      <c r="H9" s="69">
+        <v>8</v>
+      </c>
+      <c r="I9" s="69">
+        <v>9</v>
+      </c>
+      <c r="J9" s="70">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="G8" s="15"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="18"/>
-      <c r="J8" s="18"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="19">
-        <v>1</v>
-      </c>
-      <c r="B9" s="6">
-        <v>2</v>
-      </c>
-      <c r="C9" s="6">
-        <v>3</v>
-      </c>
-      <c r="D9" s="6">
-        <v>4</v>
-      </c>
-      <c r="E9" s="20">
-        <v>5</v>
-      </c>
-      <c r="F9" s="21">
-        <v>6</v>
-      </c>
-      <c r="G9" s="21">
-        <v>7</v>
-      </c>
-      <c r="H9" s="21">
-        <v>8</v>
-      </c>
-      <c r="I9" s="21">
-        <v>9</v>
-      </c>
-      <c r="J9" s="21">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="22" t="s">
+      <c r="B10" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="23" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" s="24">
+      <c r="C10" s="57">
         <f>'[1]PENDAPATAN PERBULAN'!C168</f>
         <v>170765575</v>
       </c>
-      <c r="D10" s="25">
+      <c r="D10" s="58">
         <f>'[1]BELANJA PERBULAN'!C146</f>
         <v>140690955</v>
       </c>
-      <c r="E10" s="25">
+      <c r="E10" s="58">
         <f>'[1]PENDAPATAN PERBULAN'!C182</f>
         <v>0</v>
       </c>
-      <c r="F10" s="25">
+      <c r="F10" s="58">
         <f>'[1]BELANJA PERBULAN'!C159</f>
         <v>0</v>
       </c>
-      <c r="G10" s="25">
+      <c r="G10" s="58">
         <f>D10-H10-I10</f>
         <v>139012520</v>
       </c>
-      <c r="H10" s="25">
+      <c r="H10" s="58">
         <f>'[1]BELANJA PERBULAN'!C13</f>
         <v>0</v>
       </c>
-      <c r="I10" s="25">
+      <c r="I10" s="58">
         <f>'[1]BELANJA PERBULAN'!C14</f>
         <v>1678435</v>
       </c>
-      <c r="J10" s="25">
+      <c r="J10" s="58">
         <f>'[1]BELANJA PERBULAN'!C15</f>
         <v>8106839</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="26">
+      <c r="A11" s="8">
         <f>[2]Jemaat!$B$11</f>
         <v>2069034756</v>
       </c>
-      <c r="B11" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="25">
+      <c r="B11" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="7">
         <f>'[1]PENDAPATAN PERBULAN'!D168</f>
         <v>134597000</v>
       </c>
-      <c r="D11" s="25">
+      <c r="D11" s="7">
         <f>'[1]BELANJA PERBULAN'!D146</f>
         <v>133209892</v>
       </c>
-      <c r="E11" s="25">
+      <c r="E11" s="7">
         <f>'[1]PENDAPATAN PERBULAN'!D182</f>
         <v>0</v>
       </c>
-      <c r="F11" s="25">
+      <c r="F11" s="7">
         <f>'[1]BELANJA PERBULAN'!D159</f>
         <v>0</v>
       </c>
-      <c r="G11" s="25">
+      <c r="G11" s="7">
         <f>D11-H11-I11</f>
         <v>81178418</v>
       </c>
-      <c r="H11" s="25">
+      <c r="H11" s="7">
         <f>'[1]BELANJA PERBULAN'!D13</f>
         <v>50353039</v>
       </c>
-      <c r="I11" s="25">
+      <c r="I11" s="7">
         <f>'[1]BELANJA PERBULAN'!D14</f>
         <v>1678435</v>
       </c>
-      <c r="J11" s="25">
+      <c r="J11" s="7">
         <f>'[1]BELANJA PERBULAN'!D15</f>
         <v>8106839</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="27"/>
-      <c r="B12" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="C12" s="25">
+      <c r="A12" s="9"/>
+      <c r="B12" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12" s="7">
         <f>'[1]PENDAPATAN PERBULAN'!E168</f>
         <v>183619200</v>
       </c>
-      <c r="D12" s="25">
+      <c r="D12" s="7">
         <f>'[1]BELANJA PERBULAN'!E146</f>
         <v>200967382</v>
       </c>
-      <c r="E12" s="25">
+      <c r="E12" s="7">
         <f>'[1]PENDAPATAN PERBULAN'!E182</f>
         <v>1221000</v>
       </c>
-      <c r="F12" s="25">
+      <c r="F12" s="7">
         <f>'[1]BELANJA PERBULAN'!E159</f>
         <v>1221000</v>
       </c>
-      <c r="G12" s="25">
-        <f t="shared" ref="G12:G15" si="0">D12-H12-I12</f>
+      <c r="G12" s="7">
+        <f>D12-H12-I12</f>
         <v>148937858</v>
       </c>
-      <c r="H12" s="25">
+      <c r="H12" s="7">
         <f>[2]Jemaat!$I$12</f>
         <v>50353089</v>
       </c>
-      <c r="I12" s="25">
+      <c r="I12" s="7">
         <f>[2]Jemaat!$J$12</f>
         <v>1676435</v>
       </c>
-      <c r="J12" s="25">
+      <c r="J12" s="7">
         <f>'[1]BELANJA PERBULAN'!E15</f>
         <v>8106839</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="27" t="s">
+      <c r="A13" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="C13" s="25">
+      <c r="C13" s="7">
         <f>'[1]PENDAPATAN PERBULAN'!F168</f>
         <v>183125400</v>
       </c>
-      <c r="D13" s="25">
+      <c r="D13" s="7">
         <f>'[1]BELANJA PERBULAN'!F146</f>
         <v>174740813</v>
       </c>
-      <c r="E13" s="25">
+      <c r="E13" s="7">
         <f>'[1]PENDAPATAN PERBULAN'!F182</f>
         <v>0</v>
       </c>
-      <c r="F13" s="25">
+      <c r="F13" s="7">
         <f>'[1]BELANJA PERBULAN'!F159</f>
         <v>0</v>
       </c>
-      <c r="G13" s="25">
-        <f t="shared" si="0"/>
+      <c r="G13" s="7">
+        <f t="shared" ref="G12:G14" si="0">D13-H13-I13</f>
         <v>122709339</v>
       </c>
-      <c r="H13" s="25">
+      <c r="H13" s="7">
         <f>'[1]BELANJA PERBULAN'!F13</f>
         <v>50353039</v>
       </c>
-      <c r="I13" s="25">
+      <c r="I13" s="7">
         <f>'[1]BELANJA PERBULAN'!F14</f>
         <v>1678435</v>
       </c>
-      <c r="J13" s="25">
+      <c r="J13" s="7">
         <f>'[1]BELANJA PERBULAN'!F15</f>
         <v>8106839</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="26">
+      <c r="A14" s="8">
         <f>[2]Jemaat!$B$14</f>
         <v>2069034756</v>
       </c>
-      <c r="B14" s="23" t="s">
-        <v>25</v>
-      </c>
-      <c r="C14" s="25">
+      <c r="B14" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="7">
         <f>'[1]PENDAPATAN PERBULAN'!G168</f>
         <v>160755500</v>
       </c>
-      <c r="D14" s="25">
+      <c r="D14" s="7">
         <f>'[1]BELANJA PERBULAN'!G146</f>
         <v>166555345</v>
       </c>
-      <c r="E14" s="25">
+      <c r="E14" s="7">
         <f>'[1]PENDAPATAN PERBULAN'!G182</f>
         <v>1066000</v>
       </c>
-      <c r="F14" s="25">
+      <c r="F14" s="7">
         <f>'[1]BELANJA PERBULAN'!G159</f>
         <v>1066000</v>
       </c>
-      <c r="G14" s="25">
+      <c r="G14" s="7">
         <f t="shared" si="0"/>
         <v>114523871</v>
       </c>
-      <c r="H14" s="25">
+      <c r="H14" s="7">
         <f>'[1]BELANJA PERBULAN'!G13</f>
         <v>50353039</v>
       </c>
-      <c r="I14" s="25">
+      <c r="I14" s="7">
         <f>'[1]BELANJA PERBULAN'!G14</f>
         <v>1678435</v>
       </c>
-      <c r="J14" s="25">
+      <c r="J14" s="7">
         <f>'[1]BELANJA PERBULAN'!G15</f>
         <v>8106839</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="27"/>
-      <c r="B15" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="C15" s="25">
+      <c r="A15" s="9"/>
+      <c r="B15" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15" s="7">
         <f>'[1]PENDAPATAN PERBULAN'!H168</f>
         <v>196155000</v>
       </c>
-      <c r="D15" s="25">
+      <c r="D15" s="7">
         <f>'[1]BELANJA PERBULAN'!H146</f>
         <v>176020648</v>
       </c>
-      <c r="E15" s="25">
+      <c r="E15" s="7">
         <f>'[1]PENDAPATAN PERBULAN'!H182</f>
         <v>0</v>
       </c>
-      <c r="F15" s="25">
+      <c r="F15" s="7">
         <f>'[1]BELANJA PERBULAN'!H159</f>
         <v>0</v>
       </c>
-      <c r="G15" s="25">
+      <c r="G15" s="7">
         <f>D15-H15-I15</f>
         <v>123989174</v>
       </c>
-      <c r="H15" s="25">
+      <c r="H15" s="7">
         <f>'[1]BELANJA PERBULAN'!H13</f>
         <v>50353039</v>
       </c>
-      <c r="I15" s="25">
+      <c r="I15" s="7">
         <f>'[1]BELANJA PERBULAN'!H14</f>
         <v>1678435</v>
       </c>
-      <c r="J15" s="25">
+      <c r="J15" s="7">
         <f>'[1]BELANJA PERBULAN'!H15</f>
         <v>8106839</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="27"/>
-      <c r="B16" s="23" t="s">
-        <v>27</v>
-      </c>
-      <c r="C16" s="25">
+      <c r="A16" s="9"/>
+      <c r="B16" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16" s="7">
         <f>'[1]PENDAPATAN PERBULAN'!J168</f>
         <v>148666000</v>
       </c>
-      <c r="D16" s="25">
+      <c r="D16" s="7">
         <f>'[1]BELANJA PERBULAN'!J146</f>
         <v>155593157</v>
       </c>
-      <c r="E16" s="25">
+      <c r="E16" s="7">
         <f>'[1]PENDAPATAN PERBULAN'!J182</f>
         <v>0</v>
       </c>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25">
+      <c r="F16" s="7"/>
+      <c r="G16" s="7">
         <f>D16-H16-I16</f>
         <v>103561683</v>
       </c>
-      <c r="H16" s="25">
+      <c r="H16" s="7">
         <f>'[1]BELANJA PERBULAN'!J13</f>
         <v>50353039</v>
       </c>
-      <c r="I16" s="25">
+      <c r="I16" s="7">
         <f>'[1]BELANJA PERBULAN'!J14</f>
         <v>1678435</v>
       </c>
-      <c r="J16" s="25">
+      <c r="J16" s="7">
         <f>'[1]BELANJA PERBULAN'!J15</f>
         <v>8106839</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" s="27" t="s">
+      <c r="A17" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B17" s="23" t="s">
-        <v>29</v>
-      </c>
-      <c r="C17" s="25">
+      <c r="C17" s="7">
         <f>'[1]PENDAPATAN PERBULAN'!K168</f>
         <v>182816000</v>
       </c>
-      <c r="D17" s="25">
+      <c r="D17" s="7">
         <f>'[1]BELANJA PERBULAN'!K146</f>
         <v>138890174</v>
       </c>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="28">
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="10">
         <f t="shared" ref="G17:G21" si="1">D17-H17-I17</f>
         <v>86858700</v>
       </c>
-      <c r="H17" s="25">
+      <c r="H17" s="7">
         <f>'[1]BELANJA PERBULAN'!K13</f>
         <v>50353039</v>
       </c>
-      <c r="I17" s="25">
+      <c r="I17" s="7">
         <f>'[1]BELANJA PERBULAN'!K14</f>
         <v>1678435</v>
       </c>
-      <c r="J17" s="25">
+      <c r="J17" s="7">
         <f>'[1]BELANJA PERBULAN'!K15</f>
         <v>8106839</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="27" t="s">
+      <c r="A18" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="23" t="s">
-        <v>31</v>
-      </c>
-      <c r="C18" s="25">
+      <c r="C18" s="7">
         <f>'[1]PENDAPATAN PERBULAN'!L168</f>
         <v>213422100</v>
       </c>
-      <c r="D18" s="25">
+      <c r="D18" s="7">
         <f>'[1]BELANJA PERBULAN'!L146</f>
         <v>235334402</v>
       </c>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="28">
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="10">
         <f t="shared" si="1"/>
         <v>132949889</v>
       </c>
-      <c r="H18" s="25">
+      <c r="H18" s="7">
         <f>'[1]BELANJA PERBULAN'!L13</f>
         <v>100706078</v>
       </c>
-      <c r="I18" s="25">
+      <c r="I18" s="7">
         <f>'[1]BELANJA PERBULAN'!L14</f>
         <v>1678435</v>
       </c>
-      <c r="J18" s="25">
+      <c r="J18" s="7">
         <f>'[1]BELANJA PERBULAN'!L15</f>
         <v>8106839</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="26">
+      <c r="A19" s="8">
         <f>[2]Jemaat!$B$19</f>
         <v>2014121542</v>
       </c>
-      <c r="B19" s="23" t="s">
-        <v>32</v>
-      </c>
-      <c r="C19" s="25">
+      <c r="B19" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C19" s="7">
         <f>'[1]PENDAPATAN PERBULAN'!M168</f>
         <v>197719700</v>
       </c>
-      <c r="D19" s="25">
+      <c r="D19" s="7">
         <f>'[1]BELANJA PERBULAN'!M146</f>
         <v>177457059</v>
       </c>
-      <c r="E19" s="25"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="28">
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="10">
         <f t="shared" si="1"/>
         <v>125425585</v>
       </c>
-      <c r="H19" s="25">
+      <c r="H19" s="7">
         <f>'[1]BELANJA PERBULAN'!M13</f>
         <v>50353039</v>
       </c>
-      <c r="I19" s="25">
+      <c r="I19" s="7">
         <f>'[1]BELANJA PERBULAN'!M14</f>
         <v>1678435</v>
       </c>
-      <c r="J19" s="25">
+      <c r="J19" s="7">
         <f>'[1]BELANJA PERBULAN'!M15</f>
         <v>8106839</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" s="27"/>
-      <c r="B20" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C20" s="25">
+      <c r="A20" s="9"/>
+      <c r="B20" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C20" s="7">
         <f>'[1]PENDAPATAN PERBULAN'!N168</f>
         <v>163520600</v>
       </c>
-      <c r="D20" s="25">
+      <c r="D20" s="7">
         <f>'[1]BELANJA PERBULAN'!N146</f>
         <v>194924413</v>
       </c>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="28">
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="10">
         <f t="shared" si="1"/>
         <v>142892939</v>
       </c>
-      <c r="H20" s="25">
+      <c r="H20" s="7">
         <f>'[1]BELANJA PERBULAN'!N13</f>
         <v>50353039</v>
       </c>
-      <c r="I20" s="25">
+      <c r="I20" s="7">
         <f>'[1]BELANJA PERBULAN'!N14</f>
         <v>1678435</v>
       </c>
-      <c r="J20" s="25">
+      <c r="J20" s="7">
         <f>'[1]BELANJA PERBULAN'!N15</f>
         <v>8106839</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A21" s="29"/>
-      <c r="B21" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="C21" s="25">
+      <c r="A21" s="11"/>
+      <c r="B21" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21" s="7">
         <f>'[1]PENDAPATAN PERBULAN'!O168</f>
         <v>268010800</v>
       </c>
-      <c r="D21" s="25">
+      <c r="D21" s="7">
         <f>'[1]BELANJA PERBULAN'!O146</f>
         <v>283802283</v>
       </c>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="28">
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="10">
         <f t="shared" si="1"/>
         <v>231770809</v>
       </c>
-      <c r="H21" s="25">
+      <c r="H21" s="7">
         <f>'[1]BELANJA PERBULAN'!O13</f>
         <v>50353039</v>
       </c>
-      <c r="I21" s="25">
+      <c r="I21" s="7">
         <f>'[1]BELANJA PERBULAN'!O14</f>
         <v>1678435</v>
       </c>
-      <c r="J21" s="25">
+      <c r="J21" s="7">
         <v>8106839</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="B22" s="9"/>
-      <c r="C22" s="30">
+      <c r="A22" s="34" t="s">
+        <v>34</v>
+      </c>
+      <c r="B22" s="35"/>
+      <c r="C22" s="12">
         <f>SUM(C10:C21)</f>
         <v>2203172875</v>
       </c>
-      <c r="D22" s="30">
+      <c r="D22" s="12">
         <f>SUM(D10:D21)</f>
         <v>2178186523</v>
       </c>
-      <c r="E22" s="30">
+      <c r="E22" s="12">
         <f t="shared" ref="E22:F22" si="2">SUM(E10:E21)</f>
         <v>2287000</v>
       </c>
-      <c r="F22" s="30">
+      <c r="F22" s="12">
         <f t="shared" si="2"/>
         <v>2287000</v>
       </c>
-      <c r="G22" s="30">
+      <c r="G22" s="12">
         <f>SUM(G10:G21)</f>
         <v>1553810785</v>
       </c>
-      <c r="H22" s="30">
+      <c r="H22" s="12">
         <f>SUM(H10:H21)</f>
         <v>604236518</v>
       </c>
-      <c r="I22" s="30">
+      <c r="I22" s="12">
         <f>SUM(I10:I21)</f>
         <v>20139220</v>
       </c>
-      <c r="J22" s="30">
+      <c r="J22" s="12">
         <f>SUM(J10:J21)</f>
         <v>97282068</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" s="31"/>
-      <c r="B23" s="31"/>
-      <c r="C23" s="32" t="s">
-        <v>36</v>
-      </c>
-      <c r="D23" s="30">
+      <c r="A23" s="13"/>
+      <c r="B23" s="13"/>
+      <c r="C23" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="D23" s="12">
         <f>C22-D22</f>
         <v>24986352</v>
       </c>
-      <c r="E23" s="33"/>
-      <c r="F23" s="34"/>
-      <c r="G23" s="33"/>
-      <c r="H23" s="33"/>
-      <c r="I23" s="33"/>
-      <c r="J23" s="33"/>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" s="35">
+      <c r="E23" s="15"/>
+      <c r="F23" s="16"/>
+      <c r="G23" s="15"/>
+      <c r="H23" s="15"/>
+      <c r="I23" s="15"/>
+      <c r="J23" s="15"/>
+    </row>
+    <row r="24" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="17">
         <f>A19-B31-B32</f>
         <v>1389743863.98</v>
       </c>
-      <c r="B24" s="36"/>
-      <c r="C24" s="36"/>
-      <c r="D24" s="36"/>
-      <c r="E24" s="36"/>
-      <c r="F24" s="36"/>
-      <c r="G24" s="36"/>
-      <c r="H24" s="36"/>
-      <c r="I24" s="36"/>
-      <c r="J24" s="36"/>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A25" s="6" t="s">
+      <c r="B24" s="18"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="18"/>
+      <c r="F24" s="18"/>
+      <c r="G24" s="18"/>
+      <c r="H24" s="18"/>
+      <c r="I24" s="18"/>
+      <c r="J24" s="18"/>
+    </row>
+    <row r="25" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="47" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="C25" s="48" t="s">
         <v>38</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="D25" s="49" t="s">
         <v>39</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="E25" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="E25" s="37" t="s">
+      <c r="F25" s="36"/>
+      <c r="G25" s="36"/>
+      <c r="H25" s="36"/>
+      <c r="I25" s="36"/>
+      <c r="J25" s="36"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="44" t="s">
         <v>41</v>
       </c>
-      <c r="F25" s="37"/>
-      <c r="G25" s="37"/>
-      <c r="H25" s="37"/>
-      <c r="I25" s="37"/>
-      <c r="J25" s="37"/>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A26" s="38" t="s">
-        <v>42</v>
-      </c>
-      <c r="B26" s="39">
+      <c r="B26" s="45">
         <f>B31/2</f>
         <v>302118231.30000001</v>
       </c>
-      <c r="C26" s="39">
+      <c r="C26" s="45">
         <f>H22</f>
         <v>604236518</v>
       </c>
-      <c r="D26" s="40">
+      <c r="D26" s="46">
         <f>B26-C26</f>
         <v>-302118286.69999999</v>
       </c>
-      <c r="E26" s="41"/>
-      <c r="F26" s="41"/>
-      <c r="G26" s="41"/>
-      <c r="H26" s="41"/>
-      <c r="I26" s="41"/>
-      <c r="J26" s="41"/>
+      <c r="E26" s="22"/>
+      <c r="F26" s="22"/>
+      <c r="G26" s="22"/>
+      <c r="H26" s="22"/>
+      <c r="I26" s="22"/>
+      <c r="J26" s="22"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A27" s="38" t="s">
-        <v>43</v>
-      </c>
-      <c r="B27" s="39">
+      <c r="A27" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B27" s="20">
         <f>B32/2</f>
         <v>10070607.710000001</v>
       </c>
-      <c r="C27" s="39">
+      <c r="C27" s="20">
         <f>I22</f>
         <v>20139220</v>
       </c>
-      <c r="D27" s="40">
+      <c r="D27" s="21">
         <f>B27-C27</f>
         <v>-10068612.289999999</v>
       </c>
-      <c r="E27" s="37" t="s">
+      <c r="E27" s="36" t="s">
+        <v>43</v>
+      </c>
+      <c r="F27" s="36"/>
+      <c r="G27" s="36"/>
+      <c r="H27" s="36" t="s">
         <v>44</v>
       </c>
-      <c r="F27" s="37"/>
-      <c r="G27" s="37"/>
-      <c r="H27" s="37" t="s">
+      <c r="I27" s="36"/>
+      <c r="J27" s="36"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" s="23" t="s">
         <v>45</v>
       </c>
-      <c r="I27" s="37"/>
-      <c r="J27" s="37"/>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" s="42" t="s">
-        <v>46</v>
-      </c>
-      <c r="B28" s="39">
+      <c r="B28" s="20">
         <f>B33/2</f>
         <v>48641035.239300005</v>
       </c>
-      <c r="C28" s="39">
+      <c r="C28" s="20">
         <f>J22</f>
         <v>97282068</v>
       </c>
-      <c r="D28" s="40">
+      <c r="D28" s="21">
         <f>B28-C28</f>
         <v>-48641032.760699995</v>
       </c>
-      <c r="E28" s="36"/>
-      <c r="F28" s="36"/>
-      <c r="G28" s="36"/>
-      <c r="H28" s="36"/>
-      <c r="I28" s="36"/>
-      <c r="J28" s="36"/>
-    </row>
-    <row r="29" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B29" s="43"/>
-      <c r="E29" s="44"/>
-      <c r="F29" s="44"/>
-      <c r="G29" s="44"/>
-      <c r="H29" s="44"/>
-      <c r="I29" s="44"/>
-      <c r="J29" s="44"/>
-    </row>
-    <row r="30" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="45" t="s">
-        <v>47</v>
-      </c>
-      <c r="B30" s="45" t="s">
+      <c r="E28" s="18"/>
+      <c r="F28" s="18"/>
+      <c r="G28" s="18"/>
+      <c r="H28" s="18"/>
+      <c r="I28" s="18"/>
+      <c r="J28" s="18"/>
+    </row>
+    <row r="29" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="24"/>
+      <c r="E29" s="25"/>
+      <c r="F29" s="25"/>
+      <c r="G29" s="25"/>
+      <c r="H29" s="25"/>
+      <c r="I29" s="25"/>
+      <c r="J29" s="25"/>
+    </row>
+    <row r="30" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="54" t="s">
+        <v>46</v>
+      </c>
+      <c r="B30" s="55" t="s">
+        <v>37</v>
+      </c>
+      <c r="C30" s="55" t="s">
         <v>38</v>
       </c>
-      <c r="C30" s="45" t="s">
+      <c r="D30" s="56" t="s">
         <v>39</v>
       </c>
-      <c r="D30" s="45" t="s">
-        <v>40</v>
-      </c>
-      <c r="E30" s="44"/>
-      <c r="F30" s="44"/>
-      <c r="G30" s="44"/>
-      <c r="H30" s="44"/>
-      <c r="I30" s="44"/>
-      <c r="J30" s="44"/>
+      <c r="E30" s="25"/>
+      <c r="F30" s="25"/>
+      <c r="G30" s="25"/>
+      <c r="H30" s="25"/>
+      <c r="I30" s="25"/>
+      <c r="J30" s="25"/>
     </row>
     <row r="31" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A31" s="46" t="s">
-        <v>42</v>
-      </c>
-      <c r="B31" s="47">
+      <c r="A31" s="50" t="s">
+        <v>41</v>
+      </c>
+      <c r="B31" s="51">
         <f>A19*30%</f>
         <v>604236462.60000002</v>
       </c>
-      <c r="C31" s="48">
+      <c r="C31" s="52">
         <f>C26</f>
         <v>604236518</v>
       </c>
-      <c r="D31" s="49">
+      <c r="D31" s="53">
         <f>B31-C31</f>
         <v>-55.399999976158142</v>
       </c>
-      <c r="E31" s="50" t="s">
+      <c r="E31" s="31" t="s">
+        <v>47</v>
+      </c>
+      <c r="F31" s="31"/>
+      <c r="G31" s="31"/>
+      <c r="H31" s="31" t="s">
         <v>48</v>
       </c>
-      <c r="F31" s="50"/>
-      <c r="G31" s="50"/>
-      <c r="H31" s="50" t="s">
-        <v>49</v>
-      </c>
-      <c r="I31" s="50"/>
-      <c r="J31" s="50"/>
+      <c r="I31" s="31"/>
+      <c r="J31" s="31"/>
     </row>
     <row r="32" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A32" s="46" t="s">
-        <v>43</v>
-      </c>
-      <c r="B32" s="47">
+      <c r="A32" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="B32" s="27">
         <f>A19*1%</f>
         <v>20141215.420000002</v>
       </c>
-      <c r="C32" s="48">
+      <c r="C32" s="28">
         <f>C27</f>
         <v>20139220</v>
       </c>
-      <c r="D32" s="49">
+      <c r="D32" s="29">
         <f>B32-C32</f>
         <v>1995.4200000017881</v>
       </c>
-      <c r="E32" s="44"/>
-      <c r="F32" s="44"/>
-      <c r="G32" s="44"/>
-      <c r="H32" s="44"/>
-      <c r="I32" s="44"/>
-      <c r="J32" s="44"/>
+      <c r="E32" s="25"/>
+      <c r="F32" s="25"/>
+      <c r="G32" s="25"/>
+      <c r="H32" s="25"/>
+      <c r="I32" s="25"/>
+      <c r="J32" s="25"/>
     </row>
     <row r="33" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A33" s="51" t="s">
-        <v>46</v>
-      </c>
-      <c r="B33" s="47">
+      <c r="A33" s="30" t="s">
+        <v>45</v>
+      </c>
+      <c r="B33" s="27">
         <f>A24*7%</f>
         <v>97282070.47860001</v>
       </c>
-      <c r="C33" s="48">
+      <c r="C33" s="28">
         <f>C28</f>
         <v>97282068</v>
       </c>
-      <c r="D33" s="49">
+      <c r="D33" s="29">
         <f>B33-C33</f>
         <v>2.4786000102758408</v>
       </c>
-      <c r="E33" s="44"/>
-      <c r="F33" s="44"/>
-      <c r="G33" s="44"/>
-      <c r="H33" s="44"/>
-      <c r="I33" s="44"/>
-      <c r="J33" s="44"/>
+      <c r="E33" s="25"/>
+      <c r="F33" s="25"/>
+      <c r="G33" s="25"/>
+      <c r="H33" s="25"/>
+      <c r="I33" s="25"/>
+      <c r="J33" s="25"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="18">
-    <mergeCell ref="E31:G31"/>
-    <mergeCell ref="H31:J31"/>
-    <mergeCell ref="I7:I8"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="E25:J25"/>
-    <mergeCell ref="E27:G27"/>
-    <mergeCell ref="H27:J27"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="A3:J3"/>
@@ -2084,6 +2325,14 @@
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="G7:G8"/>
     <mergeCell ref="H7:H8"/>
+    <mergeCell ref="E31:G31"/>
+    <mergeCell ref="H31:J31"/>
+    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="E25:J25"/>
+    <mergeCell ref="E27:G27"/>
+    <mergeCell ref="H27:J27"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="256" scale="85" orientation="landscape" r:id="rId1"/>

</xml_diff>